<commit_message>
Add completed reflection Q0-Q5 and full evaluation results
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/results/results_gpt4o_mini.xlsx
+++ b/results/results_gpt4o_mini.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE5"/>
+  <dimension ref="A1:AE16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -614,18 +614,18 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>I don't have access to a live database or the ability to extract current data directly. However, I can provide a list of some well-known semiconductor companies based on information available up to October 2023. Here are some prominent semiconductor companies:  1. **Intel Corporation** 2. **Samsung Electronics** 3. **Taiwan Semiconductor Manufacturing Company (TSMC)** 4. **NVIDIA Corporation** 5. **Qualcomm Incorporated** 6. **Texas Instruments** 7. **Advanced Micro Devices (AMD)** 8. **Micron Technology** 9. **Broadcom Inc.** 10. **STMicroelectronics** 11. **Infineon Technologies** 12. **Analog Devices** 13. **Marvell Technology Group** 14. **NXP Semiconductors** 15. **Skyworks Solutions** 16. **ON Semiconductor** 17. **Renesas Electronics** 18. **Kioxia Corporation** 19. **Western Digital** 20. **ASML Holding (though primarily a manufacturing equipment provider, it’s crucial for the semiconductor industry)**  This list is not exhaustive, and the semiconductor industry is vast with many more companies operating in various sectors of the market. If you need specific information about a certain company or the industry, feel free to ask!</t>
+          <t>I don't have access to a specific database of semiconductor companies or the ability to pull in real-time data. However, I can provide a list of some well-known semiconductor companies based on the information available up to October 2023. Here are some of the major players in the semiconductor industry:  1. **Intel Corporation** 2. **Samsung Electronics** 3. **Taiwan Semiconductor Manufacturing Company (TSMC)** 4. **Qualcomm Incorporated** 5. **NVIDIA Corporation** 6. **Texas Instruments** 7. **Micron Technology** 8. **Broadcom Inc.** 9. **Advanced Micro Devices (AMD)** 10. **STMicroelectronics** 11. **Analog Devices** 12. **Infineon Technologies** 13. **NXP Semiconductors** 14. **MediaTek Inc.** 15. **Renesas Electronics Corporation**  This is not an exhaustive list, as there are many other companies globally involved in semiconductor manufacturing and design. Let me know if you need more specific information or have any other questions!</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>4.43</v>
+        <v>4.71</v>
       </c>
       <c r="H2" t="n">
         <v>2</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>The answer provides a list of well-known semiconductor companies but does not include the required tickers and is not exhaustive.</t>
+          <t>The answer provides a list of well-known semiconductor companies but does not include the required tickers or mention that it lacks access to a specific database.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -635,12 +635,12 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Missing required tickers for the listed companies | List is not exhaustive as per the expected criteria</t>
+          <t>Missing required tickers for the listed companies</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Here is a list of semiconductor companies in the database:  1. **Analog Devices, Inc. (ADI)** 2. **Applied Materials, Inc. (AMAT)** 3. **Advanced Micro Devices, Inc. (AMD)** 4. **Broadcom Inc. (AVGO)** 5. **Intel Corporation (INTC)** 6. **KLA Corporation (KLAC)** 7. **Lam Research Corporation (LRCX)** 8. **Microchip Technology Incorporated (MCHP)** 9. **Monolithic Power Systems, Inc. (MPWR)** 10. **Micron Technology, Inc. (MU)** 11. **NVIDIA Corporation (NVDA)** 12. **NXP Semiconductors N.V. (NXPI)** 13. **ON Semiconductor Corporation (ON)** 14. **QUALCOMM Incorporated (QCOM)** 15. **Qorvo, Inc. (QRVO)** 16. **Skyworks Solutions, Inc. (SWKS)** 17. **Teradyne, Inc. (TER)** 18. **Texas Instruments Incorporated (TXN)**</t>
+          <t>Here is a list of semiconductor companies in the database:  1. **Analog Devices, Inc. (ADI)** 2. **Applied Materials, Inc. (AMAT)** 3. **Advanced Micro Devices, Inc. (AMD)** 4. **Broadcom Inc. (AVGO)** 5. **Intel Corporation (INTC)** 6. **KLA Corporation (KLAC)** 7. **Lam Research Corporation (LRCX)** 8. **Microchip Technology Incorporated (MCHP)** 9. **Monolithic Power Systems, Inc. (MPWR)** 10. **Micron Technology, Inc. (MU)** 11. **NVIDIA Corporation (NVDA)** 12. **NXP Semiconductors N.V. (NXPI)** 13. **ON Semiconductor Corporation (ON)** 14. **QUALCOMM Incorporated (QCOM)** 15. **Qorvo, Inc. (QRVO)** 16. **Skyworks Solutions, Inc. (SWKS)** 17. **Teradyne, Inc. (TER)** 18. **Texas Instruments Incorporated (TXN)**  Let me know if you need more information about any specific company!</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -652,14 +652,14 @@
         <v>1</v>
       </c>
       <c r="O2" t="n">
-        <v>4.47</v>
+        <v>7.34</v>
       </c>
       <c r="P2" t="n">
         <v>2</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The answer includes many correct semiconductor companies and their tickers, but it also includes some companies that are not primarily classified as semiconductor companies, such as Applied Materials and KLA.</t>
+          <t>The answer includes many correct semiconductor companies and their tickers, but it also includes some companies that are not primarily semiconductor manufacturers, such as Applied Materials and KLA.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Here is a list of semiconductor companies identified, though no financial overview data such as market cap is available for any of them:  1. **Analog Devices, Inc. (ADI)** 2. **Advanced Micro Devices, Inc. (AMD)** 3. **Broadcom Inc. (AVGO)** 4. **Intel Corporation (INTC)** 5. **Microchip Technology Incorporated (MCHP)** 6. **Monolithic Power Systems, Inc. (MPWR)** 7. **Micron Technology, Inc. (MU)** 8. **NVIDIA Corporation (NVDA)** 9. **NXP Semiconductors N.V. (NXPI)** 10. **ON Semiconductor Corporation (ON)** 11. **QUALCOMM Incorporated (QCOM)** 12. **Qorvo, Inc. (QRVO)** 13. **Skyworks Solutions, Inc. (SWKS)** 14. **Texas Instruments Incorporated (TXN)**  If you need further information or analysis on any of these companies, feel free to ask.</t>
+          <t>Here is a list of semiconductor companies in the database:  1. Analog Devices, Inc. (ADI) 2. Advanced Micro Devices, Inc. (AMD) 3. Broadcom Inc. (AVGO) 4. Intel Corporation (INTC) 5. Microchip Technology Incorporated (MCHP) 6. Monolithic Power Systems, Inc. (MPWR) 7. Micron Technology, Inc. (MU) 8. NVIDIA Corporation (NVDA) 9. NXP Semiconductors N.V. (NXPI) 10. ON Semiconductor Corporation (ON) 11. QUALCOMM Incorporated (QCOM) 12. Qorvo, Inc. (QRVO) 13. Skyworks Solutions, Inc. (SWKS) 14. Texas Instruments Incorporated (TXN)  Please note that market capitalization and sector information for these companies is currently unavailable. If you need further details or have additional questions, feel free to ask!</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -686,15 +686,15 @@
         <v>15</v>
       </c>
       <c r="W2" t="n">
-        <v>17.86</v>
+        <v>14.85</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="Y2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>The answer includes a comprehensive list of semiconductor companies with accurate tickers, meeting all required criteria.</t>
+          <t>The answer includes all required semiconductor companies and their correct tickers as specified in the criteria.</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -749,18 +749,18 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>To determine if the US stock markets are currently open, you'll need to consider the current date, time, and whether it falls on a weekday, as US stock markets (like the NYSE and NASDAQ) typically operate Monday through Friday from 9:30 AM to 4:00 PM Eastern Time. They are closed on weekends and certain holidays.   As I don’t have access to real-time information, I recommend checking a financial news website or market app to find the exact status of the stock markets at this moment.</t>
+          <t>To determine if the US stock markets are currently open, you would need to consider the current date and time, as well as the regular trading hours for major US stock exchanges. The NYSE and NASDAQ typically operate from 9:30 AM to 4:00 PM Eastern Time on regular trading days, which are Monday through Friday, excluding market holidays.  If you can provide the current date and time, I can help you determine if the markets are open or closed.</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1.95</v>
+        <v>1.87</v>
       </c>
       <c r="H3" t="n">
         <v>1</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>The answer provides general information about trading hours but fails to give the current open/closed status of the markets.</t>
+          <t>The answer provides general trading hours but fails to give a definitive open/closed status for the current moment.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -770,12 +770,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Missing current open/closed status | No specific data provided</t>
+          <t>Missing current open/closed status | Vague response asking for additional information</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>I am currently unable to check the market status due to API rate limitations. You may want to verify the market status through another source or check the regular trading hours for US stock markets, which are typically from 9:30 AM to 4:00 PM ET on weekdays.</t>
+          <t>I'm unable to check the market status at the moment due to API rate limits. However, you can check the official market hours for US stock exchanges:  - **New York Stock Exchange (NYSE)**: Open from 9:30 AM to 4:00 PM ET, Monday to Friday. - **NASDAQ**: Open from 9:30 AM to 4:00 PM ET, Monday to Friday.  If you're checking outside of these hours, the markets are closed.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -787,14 +787,14 @@
         <v>1</v>
       </c>
       <c r="O3" t="n">
-        <v>1.9</v>
+        <v>3.31</v>
       </c>
       <c r="P3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>The answer attempted to address the question but failed to provide the current open/closed status for the NYSE and NASDAQ.</t>
+          <t>The answer provides accurate trading hours for NYSE and NASDAQ but fails to confirm the current open/closed status.</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -804,12 +804,12 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Missing current market status | No specific information on NYSE or NASDAQ</t>
+          <t>Missing current market status</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Currently, I cannot check the status of the US stock markets due to API limitations. I recommend checking a financial news website for the most up-to-date information regarding whether the markets are open.</t>
+          <t>The Market Specialist is currently unable to check the status of the US stock markets due to an API limit. Therefore, it's recommended to check an alternative source for the market status.</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -821,7 +821,7 @@
         <v>1</v>
       </c>
       <c r="W3" t="n">
-        <v>5.16</v>
+        <v>5.56</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -846,7 +846,7 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>The answer does not provide any information about the current status of the US stock markets and suggests checking elsewhere without attempting to answer the question.</t>
+          <t>The answer refused to provide the required information about the market status and suggested checking an alternative source instead.</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>Complete failure to provide required data | Evasive non-answer</t>
+          <t>Complete refusal to answer the question | No relevant data provided</t>
         </is>
       </c>
     </row>
@@ -888,18 +888,18 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>I don't have real-time data access to provide the current P/E (price-to-earnings) ratio for Apple (AAPL). The P/E ratio can change frequently based on the stock price and earnings reports. To find the latest P/E ratio for Apple, I recommend checking a financial news website, a stock market app, or your brokerage account, which typically provide up-to-date stock information.</t>
+          <t>I'm unable to provide real-time data, including the current P/E ratio of Apple Inc. (AAPL), as my training only goes up until October 2023 and I do not have live data access.   To find the P/E ratio of Apple, you can check financial news websites, stock market apps, or financial statements from the company's investor relations page. The P/E ratio is calculated by dividing the current market price per share by the earnings per share (EPS).</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>2.16</v>
+        <v>1.87</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>The answer refused to provide the requested P/E ratio and did not attempt to give any numeric value, making it a complete failure.</t>
+          <t>The answer attempted to explain how to find the P/E ratio but failed to provide the required numeric value and did not meet the expected criteria.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -909,12 +909,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Refused to answer | No numeric value provided</t>
+          <t>Missing required numeric value for P/E ratio</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>I'm unable to retrieve the P/E ratio for Apple (AAPL) at the moment due to insufficient data. Please try again later or check another source.</t>
+          <t>I'm unable to retrieve the P/E ratio for Apple (AAPL) at this moment, as there seems to be no overview data available for the stock. Please try again later or check other financial sources.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -926,7 +926,7 @@
         <v>1</v>
       </c>
       <c r="O4" t="n">
-        <v>1.9</v>
+        <v>1.58</v>
       </c>
       <c r="P4" t="n">
         <v>0</v>
@@ -948,7 +948,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>I was unable to retrieve the P/E ratio for Apple Inc. (AAPL) as the overview data is currently unavailable.</t>
+          <t>I was unable to retrieve the P/E ratio or any overview data for Apple Inc. (AAPL).</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -960,7 +960,7 @@
         <v>1</v>
       </c>
       <c r="W4" t="n">
-        <v>5.77</v>
+        <v>4.92</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -995,7 +995,7 @@
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>Complete refusal to answer | No attempt to provide relevant data</t>
+          <t>Refused to answer | No data provided</t>
         </is>
       </c>
     </row>
@@ -1027,18 +1027,18 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>I'm unable to provide real-time data or the latest news sentiment for Microsoft (MSFT) as my knowledge only goes up until October 2023, and I do not have current news access. To find the most recent news sentiment for Microsoft, I recommend checking financial news websites, stock market analysis platforms, or sentiment analysis tools that aggregate and analyze news articles related to the company.</t>
+          <t>I'm unable to provide real-time data or the latest news sentiment for Microsoft (MSFT) as of October 2023. For the most current sentiment analysis, I recommend checking financial news websites, stock market analysis platforms, or social media sentiment analysis tools. These sources will provide up-to-date information on how news and market sentiment are affecting Microsoft.</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>1.7</v>
+        <v>1.28</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>The answer refused to provide any relevant information and did not attempt to address the question.</t>
+          <t>The answer refused to provide any relevant data or analysis, failing to meet the criteria for the question.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1046,10 +1046,14 @@
           <t>False</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Complete refusal to answer | No relevant data provided</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>It appears that there are currently no latest news articles available for Microsoft (MSFT) to analyze sentiment. If you need information on a specific topic or event related to Microsoft, please let me know!</t>
+          <t>There are currently no latest news articles available for Microsoft (MSFT).</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1061,14 +1065,14 @@
         <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v>1.74</v>
+        <v>1.52</v>
       </c>
       <c r="P5" t="n">
         <v>0</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>The answer completely fails to provide any news headlines or sentiment analysis for Microsoft (MSFT), which is required.</t>
+          <t>The answer completely fails to provide any news sentiment or headlines for Microsoft, which is required.</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -1078,12 +1082,12 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Missing required data points | Vague or evasive non-answer</t>
+          <t>Missing required data points</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Currently, there is no sentiment data available for Microsoft (MSFT).</t>
+          <t>There is currently no sentiment data available for Microsoft (MSFT), as no recent news headlines could be found for analysis.</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1095,7 +1099,7 @@
         <v>1</v>
       </c>
       <c r="W5" t="n">
-        <v>4.44</v>
+        <v>5.52</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
@@ -1120,7 +1124,7 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>The answer refused to provide any sentiment data or recent headlines, failing to meet the expected criteria.</t>
+          <t>The answer refused to provide any sentiment data or recent headlines, failing to meet the criteria.</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
@@ -1130,7 +1134,1524 @@
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>Complete lack of required data | Refusal to answer the question</t>
+          <t>Complete refusal to answer | No data provided</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Q05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>What is NVIDIA's stock price performance over the last month?</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Should return NVDA start price, end price, and % change for the 1-month period.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>I'm unable to provide real-time stock price data or updates on stock performance since my knowledge only goes up to October 2023, and I don't have access to live market data. To find NVIDIA's stock price performance over the last month, I recommend checking a reliable financial news website, a stock market app, or a financial platform that tracks stock prices. These sources can provide you with the most current and accurate information.</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>The answer refused to provide any data or analysis regarding NVIDIA's stock price performance, failing to meet the expected criteria.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Complete refusal to answer | No data provided</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>NVIDIA's stock price performance over the last month shows a decrease of 2.55%. The stock started at $184.96 and ended at $180.25.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>get_price_performance</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="P6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>The answer provides the start and end prices and the percentage change, but the accuracy of the numbers cannot be verified without current data.</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Potentially fabricated stock prices | Unverified percentage change</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Over the last month, NVIDIA's stock price has experienced a decline.   - **Start Price:** $184.96 - **End Price:** $180.25 - **Percentage Change:** -2.55%  This indicates a decrease in value of approximately 2.55% over the period.</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>get_price_performance</t>
+        </is>
+      </c>
+      <c r="V6" t="n">
+        <v>1</v>
+      </c>
+      <c r="W6" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="Y6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Market Specialist</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>Orchestrator+Specialists+Critic</t>
+        </is>
+      </c>
+      <c r="AB6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>All required data points are present, numbers are accurate, and conditions are met.</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Q06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Compare the 1-year price performance of AAPL, MSFT, and GOOGL. Which grew the most?</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>price_comparison</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Should fetch 1y performance for all 3 tickers, return % change for each, and identify the highest performer.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>I don’t have real-time data access or updates on financial markets, including the 1-year price performance of specific stocks like AAPL (Apple Inc.), MSFT (Microsoft Corp.), and GOOGL (Alphabet Inc.).   To compare their 1-year price performance, you would typically look at the percentage change in their stock prices from a year ago to now. You can find this information on financial news websites, stock market apps, or brokerage platforms that provide stock performance data.  If you access the most recent stock prices, you can calculate the growth by using the formula:  \[ \text{Percentage Growth} = \left( \frac{\text{Current Price} - \text{Price 1 Year Ago}}{\text{Price 1 Year Ago}} \right) \times 100 \]  Once you calculate the percentage changes for AAPL, MSFT, and GOOGL, you can easily determine which grew the most.</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>The answer refused to provide any specific data or comparisons, failing to address the question directly.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Complete refusal to answer | No data provided for comparison</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Here is the 1-year price performance comparison for AAPL, MSFT, and GOOGL:  - **Apple Inc. (AAPL)**   - Starting Price: $212.56   - Ending Price: $250.12   - Percentage Change: **17.67%**  - **Microsoft Corp. (MSFT)**   - Starting Price: $385.61   - Ending Price: $395.55   - Percentage Change: **2.58%**  - **Alphabet Inc. (GOOGL)**   - Starting Price: $164.92   - Ending Price: $302.28   - Percentage Change: **83.29%**  Among these stocks, **Alphabet Inc. (GOOGL)** grew the most with a price increase of **83.29%** over the past year.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>get_price_performance</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="P7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>The answer provides the percentage change for each ticker but includes specific numbers that may not be accurate or verifiable.</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Specific price numbers appear fabricated or unverifiable | Missing source for performance data</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Over the past year, the price performance of AAPL, MSFT, and GOOGL is as follows:  - **AAPL (Apple Inc.)**   - Start Price: $212.56   - End Price: $250.12   - Percentage Change: **17.67%**  - **MSFT (Microsoft Corporation)**   - Start Price: $385.61   - End Price: $395.55   - Percentage Change: **2.58%**  - **GOOGL (Alphabet Inc.)**   - Start Price: $164.92   - End Price: $302.28   - Percentage Change: **83.29%**  **Comparison**: - GOOGL experienced the highest growth rate at **83.29%**. - AAPL followed with a growth of **17.67%**. - MSFT had the lowest growth, increasing by **2.58%**.  In summary, GOOGL grew the most over the past year.</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>get_price_performance</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W7" t="n">
+        <v>11.69</v>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="Y7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Market Specialist</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Orchestrator+Specialists+Critic</t>
+        </is>
+      </c>
+      <c r="AB7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>The answer provides the percentage changes for all three tickers but includes specific price data that may not be accurate or verifiable.</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>Specific price data appears fabricated or unverifiable | Potential inaccuracies in percentage calculations</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Q07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Compare the P/E ratios of AAPL, MSFT, and NVDA. Which looks most expensive?</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>fundamentals</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Should return P/E ratios for all 3 tickers and identify which has the highest P/E.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>As of my last knowledge update in October 2023, I don't have access to real-time data or specific current financial figures like the P/E ratios for AAPL (Apple Inc.), MSFT (Microsoft Corporation), and NVDA (NVIDIA Corporation). However, I can explain how to compare P/E ratios and what to look for when determining which stock may be more expensive based on that metric.  **Price-to-Earnings (P/E) Ratio Explanation:** - The P/E ratio is calculated by taking the current share price of a company and dividing it by its earnings per share (EPS).  - A higher P/E ratio can indicate that a stock is more expensive relative to its earnings, possibly signaling higher growth expectations from investors.   **How to Analyze:** 1. **Gather Data**: Check reliable financial news websites, stock market apps, or investment platforms for the latest P/E ratios of AAPL, MSFT, and NVDA. 2. **Compare Ratios**: Once you have the P/E ratios, compare them:    - A stock with a significantly higher P/E ratio than its peers may be considered more expensive.    - Consider the sector's average P/E ratio, as tech companies may generally have higher P/E ratios due to growth expectations. 3. **Context Matters**: A higher P/E isn't inherently bad; it can reflect strong expected growth. Conversely, if growth projections are not met, it can lead to a stock becoming overpriced.  **Conclusion**:  Without current data, I can't definitively say which stock appears most expensive. I recommend checking a financial news service or a stock market app for up-to-date P/E ratios to make your comparison.</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>The answer provides a good explanation of P/E ratios but fails to provide the required data for AAPL, MSFT, and NVDA, making it mostly wrong.</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Missing required data points for P/E ratios</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>It seems that I am currently unable to retrieve the company overview data, including the P/E ratios, for AAPL, MSFT, and NVDA. As a result, I can't perform the comparison of their P/E ratios at this moment.  If you have any other questions or need assistance with different data, please let me know!</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>get_company_overview, get_company_overview, get_company_overview</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>The answer refused to provide any data or attempt the comparison, failing to meet the criteria.</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Complete refusal to answer | No data provided</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Currently, there is no available information on the P/E ratios for Apple Inc. (AAPL), Microsoft Corporation (MSFT), and NVIDIA Corporation (NVDA). Therefore, a comparison of their valuations based on P/E ratios cannot be made at this time.</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>get_company_overview</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>3</v>
+      </c>
+      <c r="W8" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="Y8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Fundamentals Specialist</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Orchestrator+Specialists+Critic</t>
+        </is>
+      </c>
+      <c r="AB8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>The answer refused to provide any data or attempt a comparison, failing to meet the expected criteria.</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>Complete refusal to answer | No data provided</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Q08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Which energy stocks in the database had the best 6-month performance?</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>sector_price</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Should query the DB for energy sector tickers, fetch 6-month price performance for each, and return them ranked by % change.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>I'm unable to access real-time databases or provide live data, so I can't specify which energy stocks had the best 6-month performance. However, you can find this information by checking financial news websites, stock market analysis platforms, or using investment apps that provide performance metrics for specific stocks. Look for sections on stock performance or filters for energy sector stocks to identify those with the best returns over the past six months. If you have specific stocks in mind, I can provide general information about them.</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>The answer completely fails to address the question by refusing to provide any specific data or analysis.</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Refused to answer | No specific data provided | Vague suggestions without actionable information</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Here are the energy stocks with the best 6-month performance:  1. **Texas Pacific Land Corporation (TPL)**: +73.05% 2. **Halliburton Company (HAL)**: +56.35% 3. **Targa Resources, Inc. (TRGP)**: +48.69% 4. **Valero Energy Corporation (VLO)**: +48.16% 5. **APA Corporation (APA)**: +53.59% 6. **ConocoPhillips (COP)**: +34.28% 7. **Coterra Energy Inc. (CTRA)**: +35.07% 8. **Devon Energy Corporation (DVN)**: +38.56% 9. **Diamondback Energy, Inc. (FANG)**: +37.31% 10. **EQT Corporation (EQT)**: +29.54%  These stocks showed the highest percentage price change over the last 6 months.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>get_tickers_by_sector, get_price_performance</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>2</v>
+      </c>
+      <c r="O9" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="P9" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>The answer provides a ranked list of energy stocks with their 6-month performance percentages, but lacks verification of the data source and may contain inaccuracies.</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>No source for performance data | Potential inaccuracies in percentage changes</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>The following energy stocks demonstrated the best 6-month performance based on their percentage returns:  1. **Texas Pacific Land Corporation (TPL)**    - Current Price: $531.13    - Percentage Return: 73.05%  2. **Halliburton Company (HAL)**    - Current Price: $33.69    - Percentage Return: 56.35%  3. **APA Corporation (APA)**    - Current Price: $34.47    - Percentage Return: 53.59%  4. **Targa Resources, Inc. (TRGP)**    - Current Price: $240.05    - Percentage Return: 48.69%  5. **Valero Energy Corporation (VLO)**    - Current Price: $230.59    - Percentage Return: 48.16%  6. **ConocoPhillips (COP)**    - Current Price: $121.89    - Percentage Return: 34.28%  7. **Coterra Energy Inc. (CTRA)**    - Current Price: $32.15    - Percentage Return: 35.07%  8. **Devon Energy Corporation (DVN)**    - Current Price: $46.25    - Percentage Return: 38.56%  9. **Diamondback Energy, Inc. (FANG)**    - Current Price: $182.37    - Percentage Return: 37.31%  10. **Phillips 66 (PSX)**     - Current Price: $172.74     - Percentage Return: 33.89%  Other notable mentions include: - **EQT Corporation (EQT)**: 29.54% return at $64.37 - **Occidental Petroleum Corporation (OXY)**: 28.64% return at $57.88 - **Kinder Morgan, Inc. (KMI)**: 24.62% return at $33.39 - **Marathon Petroleum Corporation (MPC)**: 26.96% return at $226.18 - **Williams Companies, Inc. (WMB)**: 27.53% return at $73.34 - **Chevron Corporation (CVX)**: 27.75% return at $196.82 - **Schlumberger N.V. (SLB)**: 30.40% return at $44.72 - **Baker Hughes Company (BKR)**: 18.24% return at $54.26 - **EOG Resources, Inc. (EOG)**: 15.85% return at $133.60  Note: Data for Hess Corporation (HES) was not available, potentially indicating it may be delisted.   In summary, Texas Pacific Land Corporation led the pack with a 73.05% return, followed by Halliburton and APA Corporation with returns of 56.35% and 53.59%, respectively.</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>get_tickers_by_sector, get_price_performance</t>
+        </is>
+      </c>
+      <c r="V9" t="n">
+        <v>2</v>
+      </c>
+      <c r="W9" t="n">
+        <v>26.29</v>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
+      <c r="Y9" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Market Specialist</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>Orchestrator+Specialists+Critic</t>
+        </is>
+      </c>
+      <c r="AB9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>The answer provides a ranked list of energy stocks with their percentage returns, but it lacks verification of the data source and may contain fabricated numbers.</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>Specific numbers provided without source | Potentially fabricated current prices</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Q09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>What is the news sentiment for Tesla (TSLA) and how has its stock moved this month?</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>sentiment</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Should return TSLA news sentiment (label + score) AND 1-month price % change from two separate tool calls.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>I do not have access to real-time data or news sentiment analysis as my knowledge was last updated in October 2023. To get the latest sentiment regarding Tesla (TSLA), I recommend checking financial news websites, stock market analysis platforms, or sentiment analysis tools that specifically evaluate news articles and social media for recent trends and insights.  For the current stock movement, you can refer to financial news platforms or stock market apps that provide real-time stock prices and historical performance data. They will help you see how Tesla's stock has moved this month.</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>The answer completely fails to provide any required data points regarding TSLA's news sentiment or stock movement.</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>No data provided | Refusal to answer | Irrelevant suggestions</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>For Tesla (TSLA), there are currently no news articles available to analyze for sentiment.  Regarding the stock's performance this month, TSLA has experienced a decline of approximately **4.73%**, moving from a start price of **$410.63** to an end price of **$391.20**.</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>get_news_sentiment, get_price_performance</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>2</v>
+      </c>
+      <c r="O10" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="P10" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>The answer provides a stock price change but fails to deliver the required news sentiment data, which is a key component of the question.</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Missing news sentiment data</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Tesla (TSLA) stock has experienced a decline of 4.73% this month, starting at a price of $410.63 and ending at $391.20. However, there is no sentiment data available for Tesla over the past month.   In summary, TSLA's stock has decreased, but sentiment analysis is not applicable at this time.</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>get_price_performance, get_news_sentiment</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>2</v>
+      </c>
+      <c r="W10" t="n">
+        <v>8.84</v>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="Y10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Market Specialist, Sentiment Specialist</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>Orchestrator+Specialists+Critic</t>
+        </is>
+      </c>
+      <c r="AB10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>The answer provides the stock movement percentage and price points accurately but fails to include the required news sentiment data.</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>Missing sentiment data</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>What are the 52-week high and low for JPMorgan (JPM) and Goldman Sachs (GS)?</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>fundamentals</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Should return 52-week high and low for both JPM and GS fetched from Alpha Vantage.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>I'm unable to provide real-time stock data or current financial figures such as the 52-week high and low for JPMorgan (JPM) and Goldman Sachs (GS) as my knowledge is based on data up to October 2023 and I don't have access to live updates or databases. To find the most accurate and up-to-date information, I recommend checking a reliable financial news website, your brokerage platform, or financial market apps.</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>The answer refused to provide the requested data and did not attempt to give any relevant information.</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Refused to answer | No data provided</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>It seems that I'm unable to retrieve the 52-week high and low data for both JPMorgan (JPM) and Goldman Sachs (GS) at the moment. The overview data for these companies is currently not available. Would you like me to try something else, or is there any other information you need?</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>get_company_overview, get_company_overview</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>2</v>
+      </c>
+      <c r="O11" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>The answer refused to provide the requested data and did not attempt to offer any relevant information.</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Refused to answer | Data unavailable without trying</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Unfortunately, the Market Specialist was unable to provide the specific 52-week high and low prices for JPMorgan (JPM) and Goldman Sachs (GS). If you need assistance with their price performance over a specific period or any other related information, please let me know!</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="Y11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>Market Specialist</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>Orchestrator+Specialists+Critic</t>
+        </is>
+      </c>
+      <c r="AB11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>The answer refused to provide the required data and did not attempt to fetch or estimate the 52-week high and low prices.</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>Complete refusal to answer | Missing required data points</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Which tech stocks dropped this month but grew this year? Return the top 3.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>multi_condition</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Should get tech tickers from DB, fetch both 1-month and year-to-date performance, filter for negative 1-month AND positive YTD, return top 3 by yearly growth with exact percentages. Results must satisfy both conditions simultaneously.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>I'm unable to provide real-time data or specific stock performance for the current month, as my information only goes up until October 2023 and I don't have live market data. However, I can suggest a general approach for finding this information:  1. **Financial News Websites**: Websites like Bloomberg, CNBC, and Yahoo Finance frequently report on stock performance and can provide monthly analyses. 2. **Stock Market Apps**: Apps like Robinhood or MarketWatch often allow you to filter stocks based on performance over different time frames. 3. **Stock Screeners**: Tools such as Finviz or Yahoo Finance's stock screener can help you sort stocks by performance metrics.  Generally, the tech sector often has volatile movements, and it’s common for certain stocks to experience monthly declines while still posting strong gains over a longer time frame like a year. Look for stocks that are gaining attention but may have faced short-term hurdles in the current month.</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>The answer does not provide any specific stock tickers or performance data, failing to address the question directly.</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>No specific stock tickers provided | No performance data given | Vague suggestions instead of concrete answers</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Here are the top 3 technology stocks that have dropped in price this month but have shown growth this year:  1. **Advanced Micro Devices, Inc. (AMD)**    - **1 Month Change:** -4.77%    - **Year-to-Date Change:** -13.46%  2. **Amphenol Corporation (APH)**    - **1 Month Change:** -9.86%    - **Year-to-Date Change:** -4.14%     3. **Corning Incorporated (GLW)**    - **1 Month Change:** -0.89%    - **Year-to-Date Change:** +42.67%  These companies have experienced declines this month while maintaining or growing their annual performance.</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>get_tickers_by_sector, get_price_performance, get_price_performance</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>3</v>
+      </c>
+      <c r="O12" t="n">
+        <v>30.84</v>
+      </c>
+      <c r="P12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>The answer attempted to provide relevant stocks but failed to meet the criteria of having positive year-to-date growth for all listed stocks, and included incorrect data for AMD and APH.</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Incorrect year-to-date performance for AMD and APH | Only one stock (GLW) meets the criteria</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>The top three technology stocks that have experienced a decline in price this month but have shown growth over the past year are:  1. **Analog Devices, Inc. (ADI)**    - **1-Month Price Change:** -9.03%    - **Year-to-Date Price Change:** +12.16%  2. **Akamai Technologies, Inc. (AKAM)**    - **1-Month Price Change:** -0.69%    - **Year-to-Date Price Change:** +26.52%  3. **Applied Materials, Inc. (AMAT)**    - **1-Month Price Change:** -4.78%    - **Year-to-Date Price Change:** +27.18%  These stocks have demonstrated resilience, maintaining positive year-to-date performance despite recent monthly declines.   Note: No data was retrieved regarding Apple Inc. (AAPL), Microsoft Corporation (MSFT), or NVIDIA Corporation (NVDA) from the fundamentals specialist.</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>get_tickers_by_sector, get_price_performance, get_company_overview</t>
+        </is>
+      </c>
+      <c r="V12" t="n">
+        <v>7</v>
+      </c>
+      <c r="W12" t="n">
+        <v>38.8</v>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
+      <c r="Y12" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>Market Specialist, Fundamentals Specialist</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>Orchestrator+Specialists+Critic</t>
+        </is>
+      </c>
+      <c r="AB12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>The answer provides accurate tickers, correct performance percentages, and meets the criteria of negative 1-month and positive YTD growth.</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Which large-cap technology stocks on NASDAQ have grown more than 20% this year?</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>multi_condition</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Should query DB for large-cap NASDAQ tech stocks, fetch YTD performance, filter for &gt;20% growth, and return matching tickers with exact % change.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>As of my last update in October 2023, I don't have real-time data access to provide you with specific large-cap technology stocks that have grown more than 20% during the year. Stock performance can vary significantly based on market conditions, earnings reports, and other factors.   To find the most current large-cap technology stocks on NASDAQ that have grown more than 20% this year, I recommend checking a reliable financial news website, a stock market app, or using financial analysis tools such as Bloomberg, Yahoo Finance, or Google Finance. These platforms often provide performance metrics and allow you to filter stocks by various criteria, including market capitalization and year-to-date performance.</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>The answer refused to provide any specific data or analysis, failing to address the question directly.</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Complete refusal to answer | No specific data provided | Vague recommendations instead of concrete information</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>It appears that there are no large-cap technology stocks listed on NASDAQ in the local database. Therefore, I can't provide details about their performance this year. If you have any other requests or specific criteria, feel free to let me know!</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>query_local_db</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>The answer refused to provide any information and did not attempt to query or analyze data, resulting in a complete failure to address the question.</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Refusal to answer | No attempt to provide relevant data</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>As of 2023, several large-cap technology stocks on NASDAQ have experienced significant growth, each exceeding 20% year-to-date. Here are the details:  1. **Akamai Technologies, Inc. (AKAM)**    - Year-to-Date Price Change: **+26.52%**    - Start Price: $85.10    - End Price: $107.67  2. **Applied Materials, Inc. (AMAT)**    - Year-to-Date Price Change: **+27.18%**    - Start Price: $268.54    - End Price: $341.53  3. **Keysight Technologies Inc. (KEYS)**    - Year-to-Date Price Change: **+35.43%**    - Start Price: $206.59    - End Price: $279.78  4. **Micron Technology, Inc. (MU)**    - Year-to-Date Price Change: **+35.10%**    - Start Price: $315.42    - End Price: $426.13  5. **Seagate Technology Holdings PLC (STX)**    - Year-to-Date Price Change: **+33.45%**    - Start Price: $287.54    - End Price: $383.71  6. **Teradyne, Inc. (TER)**    - Year-to-Date Price Change: **+38.05%**    - Start Price: $207.47    - End Price: $286.42  7. **Western Digital Corporation (WDC)**    - Year-to-Date Price Change: **+45.14%**    - Start Price: $187.61    - End Price: $272.29  While specific financial metrics such as P/E ratios and market caps were not available, these stocks have shown robust performance in 2023. If you need further details or analysis, feel free to ask!</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>get_tickers_by_sector, get_price_performance, query_local_db, get_company_overview</t>
+        </is>
+      </c>
+      <c r="V13" t="n">
+        <v>86</v>
+      </c>
+      <c r="W13" t="n">
+        <v>56.97</v>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+      <c r="Y13" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>Market Specialist, Fundamentals Specialist</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>Orchestrator+Specialists+Critic</t>
+        </is>
+      </c>
+      <c r="AB13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>The answer provides a list of stocks with their year-to-date performance, but lacks verification of the companies being large-cap NASDAQ tech stocks and does not include P/E ratios or market caps as mentioned in the criteria.</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>Missing verification of large-cap status | Lack of P/E ratios and market caps</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>For the top 3 semiconductor stocks by 1-year return, what are their P/E ratios and current news sentiment?</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>cross_domain</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Should find semiconductor tickers in DB, rank by 1-year return to find top 3, then fetch P/E ratio AND news sentiment for each — requiring three separate data domains (price, fundamentals, sentiment).</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>I don't have real-time data or news updates as my training only includes information up to October 2023. For the most current information regarding the top semiconductor stocks by 1-year return, their P/E ratios, and current news sentiment, I recommend checking a finance news website, a stock analysis platform, or a trading app that provides real-time financial data.  To find the top semiconductor stocks by 1-year return, you can look at financial news aggregators or stock screening tools, and they typically provide the most updated P/E ratios as well as sentiment analysis based on recent news articles and social media activity. If you have any other questions or need guidance on how to analyze stocks, feel free to ask!</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>The answer completely fails to provide any specific data or attempt to answer the question, instead deflecting to external sources.</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Refusal to provide data | No attempt to answer the question</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>The top 3 semiconductor stocks by 1-year return are:  1. **Applied Materials, Inc. (AMAT)**      - **1-Year Return:** 121.37%    - **P/E Ratio:** Data not available      - **News Sentiment:** No recent articles found  2. **Lam Research Corporation (LRCX)**      - **1-Year Return:** 171.64%    - **P/E Ratio:** Data not available      - **News Sentiment:** No recent articles found  3. **Micron Technology, Inc. (MU)**      - **1-Year Return:** 324.18%    - **P/E Ratio:** Data not available      - **News Sentiment:** No recent articles found  Unfortunately, it appears that I was unable to retrieve the P/E ratios for these stocks, and there are no recent news articles available for sentiment analysis either.</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>get_tickers_by_sector, get_price_performance, get_company_overview, get_company_overview, get_company_overview, get_news_sentiment, get_news_sentiment, get_news_sentiment</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>8</v>
+      </c>
+      <c r="O14" t="n">
+        <v>8.65</v>
+      </c>
+      <c r="P14" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>The answer provides the correct stocks and their 1-year returns but fails to provide P/E ratios and news sentiment, which are required data points.</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Missing P/E ratios | Missing news sentiment</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Based on the latest data, here are the top three semiconductor stocks by 1-year return, along with their current prices and P/E ratios:  1. **Micron Technology, Inc. (MU)**    - **1-Year Return**: 324.18%    - **Current Price**: $426.13    - **P/E Ratio**: Not available  2. **Teradyne, Inc. (TER)**    - **1-Year Return**: 231.43%    - **Current Price**: $286.42    - **P/E Ratio**: Not available  3. **Lam Research Corporation (LRCX)**    - **1-Year Return**: 171.64%    - **Current Price**: $212.20    - **P/E Ratio**: Not available  Unfortunately, there is no available news sentiment data for these stocks at this time, which limits the ability to assess current market sentiment.  In summary, while the top three semiconductor stocks have shown impressive returns over the past year, P/E ratios and sentiment data are currently unavailable.</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>get_tickers_by_sector, get_price_performance, get_company_overview, query_local_db, get_news_sentiment</t>
+        </is>
+      </c>
+      <c r="V14" t="n">
+        <v>12</v>
+      </c>
+      <c r="W14" t="n">
+        <v>25.71</v>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
+      <c r="Y14" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>Market Specialist, Fundamentals Specialist, Sentiment Specialist</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>Orchestrator+Specialists+Critic</t>
+        </is>
+      </c>
+      <c r="AB14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>The answer provides some relevant data but fails to include P/E ratios and news sentiment, which are required, and the prices appear fabricated.</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>Missing P/E ratios | Missing news sentiment | Prices appear fabricated</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Compare the market cap, P/E ratio, and 1-year stock performance of JPM, GS, and BAC.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>cross_domain</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Should return market cap, P/E, and 1-year % change for all 3 tickers, combining Alpha Vantage fundamentals and yfinance price data.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>As of October 2023, I can’t provide real-time financial data, including the current market cap, P/E ratio, or 1-year stock performance for JPMorgan Chase (JPM), Goldman Sachs (GS), and Bank of America (BAC). However, I can explain how to find this information and what it generally means.  1. **Market Cap**: This is the total market value of a company's outstanding shares, calculated by multiplying the current share price by the total number of outstanding shares. You can find current market cap data on financial news websites or stock market apps.  2. **P/E Ratio**: The Price-to-Earnings (P/E) ratio is a valuation ratio calculated by dividing the market price per share by the earnings per share (EPS). A high P/E ratio may indicate that a company is overvalued, whereas a low P/E might suggest undervaluation. This information is often available on financial analysis platforms or brokerage websites.  3. **1-Year Stock Performance**: This metric reflects how much the stock price has changed over the past year. You can assess this by looking at historical stock price data, which is also found on various financial websites.   To get the latest and accurate numbers on JPM, GS, and BAC regarding market cap, P/E ratio, and stock performance, I recommend checking reputable financial news sources, stock market analysis websites like Yahoo Finance, Google Finance, or your brokerage's research section.</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>The answer fails to provide any specific data points for market cap, P/E ratio, or 1-year stock performance, and instead offers vague guidance on how to find the information.</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Missing required data points for JPM, GS, and BAC | Vague non-answer without specific figures</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>It seems I encountered an error retrieving the fundamental data (market cap and P/E ratio) for JPM, GS, and BAC. However, I was able to gather the 1-year stock performance data for these banks. Here is the performance information:  - **JPM (JPMorgan Chase)**   - **1-Year Performance:** +24.44%   - **Start Price:** $227.77   - **End Price:** $283.44  - **GS (Goldman Sachs)**   - **1-Year Performance:** +47.47%   - **Start Price:** $530.42   - **End Price:** $782.21  - **BAC (Bank of America)**   - **1-Year Performance:** +16.83%   - **Start Price:** $39.99   - **End Price:** $46.72  Unfortunately, I cannot provide the market cap or P/E ratio at this time. If you need further information or a different analysis, please let me know!</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>get_company_overview, get_company_overview, get_company_overview, get_price_performance</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>4</v>
+      </c>
+      <c r="O15" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="P15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>The answer provided the 1-year stock performance data but failed to include the required market cap and P/E ratio, which are essential for a complete comparison.</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Missing market cap and P/E ratio data</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>### Comparison of JPMorgan Chase (JPM), Goldman Sachs (GS), and Bank of America (BAC)  #### 1-Year Stock Performance - **JPMorgan Chase (JPM)**   - Start Price: $227.77   - End Price: $283.44   - Percentage Change: **+24.44%**  - **Goldman Sachs (GS)**   - Start Price: $530.42   - End Price: $782.21   - Percentage Change: **+47.47%**  - **Bank of America (BAC)**   - Start Price: $39.99   - End Price: $46.72   - Percentage Change: **+16.83%**  #### Market Capitalization and P/E Ratio Unfortunately, there is no available data regarding the market capitalization or P/E ratio for JPMorgan Chase (JPM), Goldman Sachs (GS), or Bank of America (BAC) at this time.  ### Summary In terms of 1-year stock performance, Goldman Sachs leads with a **+47.47%** increase, followed by JPMorgan Chase at **+24.44%**, and Bank of America at **+16.83%**. However, market cap and P/E ratio data are currently unavailable for all three companies.</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>get_price_performance, get_company_overview</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>4</v>
+      </c>
+      <c r="W15" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="Y15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>Market Specialist, Fundamentals Specialist</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>Orchestrator+Specialists+Critic</t>
+        </is>
+      </c>
+      <c r="AB15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>The answer provides 1-year stock performance data but fails to include market cap and P/E ratio, which are required data points.</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>Missing market cap data | Missing P/E ratio data</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Which finance sector stocks are trading closer to their 52-week low than their 52-week high? Return the news sentiment for each.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>multi_condition</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Should get finance sector tickers from DB, fetch 52-week high and low for each, compute proximity to the low, then fetch news sentiment for qualifying stocks.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>I don't have real-time data access, including current stock prices, 52-week highs/lows, or news sentiment analysis. However, I can guide you on how to find this information.  To identify finance sector stocks trading closer to their 52-week low than their 52-week high, you can use a stock screening tool, which is available on financial news websites (like Yahoo Finance, Google Finance, or Bloomberg). Here's how you could proceed:  1. **Stock Screener**: Use a stock screener that allows you to filter by sector (Finance) and set criteria for stock price compared to the 52-week range.  2. **Calculate Proximity**: For each stock, calculate how close the current price is to the 52-week low versus the 52-week high. This can be done using the following formula:    - If Current Price &lt; Midpoint of 52-Week Range (which is (52-week high + 52-week low) / 2), then it’s closer to the low.  3. **News Sentiment**: For news sentiment, you can check financial news aggregators or use sentiment analysis tools that analyze headlines and articles for positive, negative, or neutral sentiment regarding specific stocks.  4. **Additional Resources**: Websites like MarketWatch or Seeking Alpha also provide sentiment scoring based on recent articles and analyst ratings.  Remember to check multiple sources to verify the information you gather. If you're looking for specific names of stocks or precise data, financial news channels or market platforms might provide you with the most accurate and current information.</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>The answer does not provide any specific data or stock tickers, and it fails to attempt to answer the question directly.</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>No specific stock tickers provided | No 52-week high/low data mentioned | No news sentiment analysis included</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>It appears that I was unable to retrieve the necessary company overview data for any of the stocks in the Financial Services sector. This data typically includes critical figures such as the 52-week high and low, which are needed to determine which stocks are closer to their 52-week low.  As a result, I cannot provide the requested analysis of which financial sector stocks are trading closer to their 52-week low than to their 52-week high.  If you'd like to explore another option or a different sector, please let me know!</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>get_tickers_by_sector, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview, get_company_overview</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>68</v>
+      </c>
+      <c r="O16" t="n">
+        <v>24.75</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>The answer completely fails to provide any relevant data or analysis regarding the finance sector stocks as requested.</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Refused to answer | No data provided | Irrelevant suggestions for other sectors</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Currently, there are no stocks listed in the finance sector that are trading closer to their 52-week low than their 52-week high. Consequently, there is also no news sentiment available for any finance sector stocks at this time.</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>get_tickers_by_sector, query_local_db</t>
+        </is>
+      </c>
+      <c r="V16" t="n">
+        <v>2</v>
+      </c>
+      <c r="W16" t="n">
+        <v>8.81</v>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="Y16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>Market Specialist, Sentiment Specialist</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>Orchestrator+Specialists+Critic</t>
+        </is>
+      </c>
+      <c r="AB16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>The answer is a complete failure as it does not provide any relevant data or analysis regarding finance sector stocks and their proximity to 52-week highs and lows.</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>No data provided | No analysis or computation performed | Irrelevant conclusion</t>
         </is>
       </c>
     </row>
@@ -1197,16 +2718,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="E2" t="n">
-        <v>25</v>
+        <v>26.7</v>
       </c>
       <c r="F2" t="n">
-        <v>2.6</v>
+        <v>2.3</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -1224,16 +2745,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>6.7</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>2.9</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -1251,7 +2772,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -1260,7 +2781,7 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>3.1</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -1278,16 +2799,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="D5" t="n">
-        <v>0.75</v>
+        <v>0.33</v>
       </c>
       <c r="E5" t="n">
-        <v>25</v>
+        <v>11.1</v>
       </c>
       <c r="F5" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -1305,19 +2826,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>0.75</v>
+        <v>1.2</v>
       </c>
       <c r="E6" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="F6" t="n">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -1332,19 +2853,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -1359,19 +2880,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>14.3</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1386,19 +2907,19 @@
         </is>
       </c>
       <c r="C9" t="n">
+        <v>15</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="E9" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G9" t="n">
         <v>4</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E9" t="n">
-        <v>25</v>
-      </c>
-      <c r="F9" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1413,16 +2934,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D10" t="n">
-        <v>0.75</v>
+        <v>1.2</v>
       </c>
       <c r="E10" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="F10" t="n">
-        <v>8.300000000000001</v>
+        <v>7.6</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -1440,19 +2961,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>11.8</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -1467,19 +2988,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>46.7</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>28.8</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1494,19 +3015,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="D13" t="n">
-        <v>0.75</v>
+        <v>1.27</v>
       </c>
       <c r="E13" t="n">
-        <v>25</v>
+        <v>42.2</v>
       </c>
       <c r="F13" t="n">
-        <v>8.300000000000001</v>
+        <v>16.1</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>